<commit_message>
TS26 final changes June 13 24
</commit_message>
<xml_diff>
--- a/TestData/LV_TS02_PostUpdatingDFFFieldsOfOpportunity.xlsx
+++ b/TestData/LV_TS02_PostUpdatingDFFFieldsOfOpportunity.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9C3AA8C-0E39-4D03-A9C5-F504833E3D49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AD96900-A4B7-40CB-B86A-58F9F4A69924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="2" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="116">
   <si>
     <t>Client</t>
   </si>
@@ -376,6 +376,21 @@
   </si>
   <si>
     <t>James Craven</t>
+  </si>
+  <si>
+    <t>ContractName</t>
+  </si>
+  <si>
+    <t>Test Contract</t>
+  </si>
+  <si>
+    <t>Test Enterprises, Inc.</t>
+  </si>
+  <si>
+    <t>Additional Contract</t>
+  </si>
+  <si>
+    <t>ContractName2</t>
   </si>
 </sst>
 </file>
@@ -730,14 +745,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
-    <col min="3" max="3" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>19</v>
       </c>
@@ -748,7 +763,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>110</v>
       </c>
@@ -759,12 +774,12 @@
         <v>101</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>63</v>
       </c>
@@ -777,17 +792,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38D6E192-2E02-4317-8F8C-DDC04F9EC4B0}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>103</v>
       </c>
@@ -800,22 +815,22 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C19CAC9-07D1-49FB-9590-44047C1B7D24}">
   <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>107</v>
       </c>
@@ -828,34 +843,34 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AB4"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="8" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.44140625" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="8" style="4" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="21" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="27" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="11" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" customWidth="1"/>
+    <col min="26" max="26" width="11.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -941,7 +956,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>53</v>
       </c>
@@ -1027,7 +1042,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>53</v>
       </c>
@@ -1113,7 +1128,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>53</v>
       </c>
@@ -1208,18 +1223,18 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>70</v>
       </c>
@@ -1245,7 +1260,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>71</v>
       </c>
@@ -1280,14 +1295,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBC2026B-771C-414C-A779-27E02A4A364D}">
   <dimension ref="A1:G25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="30.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="126" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>79</v>
       </c>
@@ -1295,7 +1310,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>80</v>
       </c>
@@ -1303,7 +1318,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>79</v>
       </c>
@@ -1311,7 +1326,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>83</v>
       </c>
@@ -1319,7 +1334,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>80</v>
       </c>
@@ -1327,7 +1342,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>79</v>
       </c>
@@ -1335,7 +1350,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>83</v>
       </c>
@@ -1343,7 +1358,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>80</v>
       </c>
@@ -1351,7 +1366,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>79</v>
       </c>
@@ -1359,7 +1374,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
         <v>83</v>
       </c>
@@ -1367,7 +1382,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
         <v>80</v>
       </c>
@@ -1382,17 +1397,17 @@
         <v>520</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
         <v>80</v>
       </c>
@@ -1400,7 +1415,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>79</v>
       </c>
@@ -1408,7 +1423,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="7" t="s">
         <v>83</v>
       </c>
@@ -1416,7 +1431,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
         <v>80</v>
       </c>
@@ -1424,22 +1439,22 @@
         <v>82</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="6" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>90</v>
       </c>
@@ -1447,7 +1462,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>91</v>
       </c>
@@ -1455,7 +1470,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>89</v>
       </c>
@@ -1463,7 +1478,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C25" t="s">
         <v>97</v>
       </c>
@@ -1475,18 +1490,21 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>34</v>
       </c>
@@ -1511,8 +1529,17 @@
       <c r="H1" s="1" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>54</v>
       </c>
@@ -1536,6 +1563,15 @@
       </c>
       <c r="H2" t="s">
         <v>78</v>
+      </c>
+      <c r="I2" t="s">
+        <v>112</v>
+      </c>
+      <c r="J2" t="s">
+        <v>113</v>
+      </c>
+      <c r="K2" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -1547,14 +1583,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>55</v>
       </c>
@@ -1565,7 +1601,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>64</v>
       </c>

</xml_diff>